<commit_message>
Add the shared helper kit (ENH-12) and move duplicated helpers into it
DigitalSecretary.Kit holds pure, contract-free helpers several features
need: ByteSize, PauseToken, FileBytes, GrayImage/ImageHasher and the
undo-able ReviewFolder mover. A feature opts in with <UseKit>true</UseKit>;
the kit DLL ships inside that feature's plugin folder and loads in its own
PluginLoadContext, so the host never references it and features remain
independent. Removes three copies of ByteSize/PauseToken and their four
duplicate test files. Similar Pictures' ReviewMover keeps its keeper rule
and delegates the moving and undo to the kit. Golden rule 1, the coding
standards and the architecture doc describe the exception.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/traceability/DigitalSecretary-Traceability-Matrix.xlsx
+++ b/docs/traceability/DigitalSecretary-Traceability-Matrix.xlsx
@@ -5071,7 +5071,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>src/Features/DeDupeFiles/DeDupeReportText.cs (Render), src/Features/DeDupeFiles/ByteSize.cs (Format)</t>
+          <t>src/Features/DeDupeFiles/DeDupeReportText.cs (Render), src/DigitalSecretary.Kit/ByteSize.cs (Format)</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -5133,12 +5133,12 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>src/Features/DeDupeFiles/PauseToken.cs (Pause, Resume), src/Features/DeDupeFiles/DeDupeFilesControl.cs (OnPauseResume, OnStop)</t>
+          <t>src/DigitalSecretary.Kit/PauseToken.cs (Pause, Resume), src/Features/DeDupeFiles/DeDupeFilesControl.cs (OnPauseResume, OnStop)</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>tests/DigitalSecretary.UnitTests/Features/DeDupeFiles/PauseTokenTests.cs</t>
+          <t>tests/DigitalSecretary.UnitTests/Kit/PauseTokenTests.cs</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -6249,12 +6249,12 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>src/Features/SimilarPictures/GrayImage.cs (Resize, Transform, LaplacianVariance)</t>
+          <t>src/DigitalSecretary.Kit/GrayImage.cs (Resize, Transform, LaplacianVariance)</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>tests/DigitalSecretary.UnitTests/Features/SimilarPictures/GrayImageTests.cs</t>
+          <t>tests/DigitalSecretary.UnitTests/Kit/GrayImageTests.cs</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -6311,7 +6311,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>src/Features/SimilarPictures/ImageHasher.cs (Compute, PerceptualHash, DifferenceHash)</t>
+          <t>src/DigitalSecretary.Kit/ImageHasher.cs (Compute, PerceptualHash, DifferenceHash)</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>src/Features/SimilarPictures/ReviewMover.cs (Plan, Run, TargetFor)</t>
+          <t>src/Features/SimilarPictures/ReviewMover.cs (Plan, Run, TargetFor), src/DigitalSecretary.Kit/ReviewFolder.cs (Run, TargetFor)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>src/Features/SimilarPictures/ReviewMover.cs (Undo, SaveLastBatch, LoadLastBatch)</t>
+          <t>src/Features/SimilarPictures/ReviewMover.cs (Undo, SaveLastBatch, LoadLastBatch), src/DigitalSecretary.Kit/ReviewFolder.cs (Undo, SaveLastBatch, LoadLastBatch)</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">

</xml_diff>